<commit_message>
IDEFICS-5: changing sodium variable and the physical activity + all other changes that were only present in the idefics repo
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_proc_elem/DPE_IDEFICS_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_proc_elem/DPE_IDEFICS_FRANZI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Projekte\NFDI4Health\TA5\Pilotprojekte\Harmonisierung\HarmonizR\use-cases-harmonisation\analyst\Franzi\rmonize\data_proc_elem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Franzi\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{68140089-BBF9-486E-BCD1-79260BE80421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0315D801-E0A7-4EFC-A698-B29C5EB2EBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -849,9 +849,6 @@
     <t>IDEFICS_P1</t>
   </si>
   <si>
-    <t>_BLANK_</t>
-  </si>
-  <si>
     <t>paste</t>
   </si>
   <si>
@@ -1857,6 +1854,9 @@
       </rPr>
       <t xml:space="preserve"> SACANA FGS L47 "Based on potatoes")</t>
     </r>
+  </si>
+  <si>
+    <t>__BLANK__</t>
   </si>
 </sst>
 </file>
@@ -2362,7 +2362,7 @@
         <v>253</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J2" s="7" t="s">
         <v>254</v>
@@ -2396,7 +2396,7 @@
         <v>253</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>254</v>
@@ -2461,7 +2461,7 @@
         <v>253</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>254</v>
@@ -2494,7 +2494,7 @@
         <v>253</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J6" s="16" t="s">
         <v>254</v>
@@ -2526,7 +2526,7 @@
         <v>253</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J7" s="16" t="s">
         <v>254</v>
@@ -2558,7 +2558,7 @@
         <v>253</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>254</v>
@@ -2590,7 +2590,7 @@
         <v>253</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J9" s="16" t="s">
         <v>254</v>
@@ -2622,7 +2622,7 @@
         <v>253</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="J10" s="16" t="s">
         <v>254</v>
@@ -2654,7 +2654,7 @@
         <v>253</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J11" s="16" t="s">
         <v>254</v>
@@ -2686,7 +2686,7 @@
         <v>253</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>254</v>
@@ -2718,7 +2718,7 @@
         <v>253</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>254</v>
@@ -2750,7 +2750,7 @@
         <v>253</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>254</v>
@@ -2782,7 +2782,7 @@
         <v>253</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J15" s="12" t="s">
         <v>254</v>
@@ -2844,7 +2844,7 @@
         <v>253</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>254</v>
@@ -2941,7 +2941,7 @@
         <v>253</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>254</v>
@@ -2974,7 +2974,7 @@
         <v>253</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>254</v>
@@ -3007,7 +3007,7 @@
         <v>253</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J22" s="12" t="s">
         <v>254</v>
@@ -3136,7 +3136,7 @@
         <v>253</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J26" s="12" t="s">
         <v>254</v>
@@ -3169,7 +3169,7 @@
         <v>253</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J27" s="12" t="s">
         <v>254</v>
@@ -3201,7 +3201,7 @@
         <v>253</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J28" s="12" t="s">
         <v>254</v>
@@ -3377,7 +3377,7 @@
         <v>253</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>254</v>
@@ -3440,7 +3440,7 @@
         <v>253</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J35" s="12" t="s">
         <v>254</v>
@@ -3473,7 +3473,7 @@
         <v>253</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J36" s="12" t="s">
         <v>254</v>
@@ -3506,7 +3506,7 @@
         <v>253</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J37" s="12" t="s">
         <v>254</v>
@@ -3539,7 +3539,7 @@
         <v>253</v>
       </c>
       <c r="I38" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>254</v>
@@ -3572,7 +3572,7 @@
         <v>253</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="J39" s="12" t="s">
         <v>254</v>
@@ -3605,7 +3605,7 @@
         <v>253</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>254</v>
@@ -3668,7 +3668,7 @@
         <v>253</v>
       </c>
       <c r="I42" s="15" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J42" s="15" t="s">
         <v>254</v>
@@ -3701,7 +3701,7 @@
         <v>253</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J43" s="3" t="s">
         <v>254</v>
@@ -3734,7 +3734,7 @@
         <v>253</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J44" s="3" t="s">
         <v>254</v>
@@ -3767,7 +3767,7 @@
         <v>253</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J45" s="3" t="s">
         <v>254</v>
@@ -3800,7 +3800,7 @@
         <v>253</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J46" s="3" t="s">
         <v>254</v>
@@ -3833,7 +3833,7 @@
         <v>253</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J47" s="3" t="s">
         <v>254</v>
@@ -3927,7 +3927,7 @@
         <v>253</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J50" s="3" t="s">
         <v>254</v>
@@ -3990,7 +3990,7 @@
         <v>253</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J52" s="3" t="s">
         <v>254</v>
@@ -4023,7 +4023,7 @@
         <v>253</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J53" s="3" t="s">
         <v>254</v>
@@ -4056,7 +4056,7 @@
         <v>253</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J54" s="3" t="s">
         <v>254</v>
@@ -4182,7 +4182,7 @@
         <v>253</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J58" s="3" t="s">
         <v>254</v>
@@ -4247,7 +4247,7 @@
         <v>253</v>
       </c>
       <c r="I60" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J60" s="12" t="s">
         <v>254</v>
@@ -4280,7 +4280,7 @@
         <v>253</v>
       </c>
       <c r="I61" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J61" s="7" t="s">
         <v>254</v>
@@ -4313,7 +4313,7 @@
         <v>253</v>
       </c>
       <c r="I62" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J62" s="7" t="s">
         <v>254</v>
@@ -4378,7 +4378,7 @@
         <v>253</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J64" s="15" t="s">
         <v>254</v>
@@ -4442,7 +4442,7 @@
         <v>253</v>
       </c>
       <c r="I66" s="7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J66" s="7" t="s">
         <v>254</v>
@@ -4474,7 +4474,7 @@
         <v>253</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J67" s="3" t="s">
         <v>254</v>
@@ -4506,7 +4506,7 @@
         <v>253</v>
       </c>
       <c r="I68" s="12" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J68" s="12" t="s">
         <v>254</v>
@@ -4662,7 +4662,7 @@
         <v>253</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J73" s="3" t="s">
         <v>254</v>
@@ -4726,7 +4726,7 @@
         <v>253</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J75" s="3" t="s">
         <v>254</v>
@@ -4758,7 +4758,7 @@
         <v>253</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>254</v>
@@ -4820,7 +4820,7 @@
         <v>253</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J78" s="3" t="s">
         <v>254</v>
@@ -4853,10 +4853,10 @@
         <v>253</v>
       </c>
       <c r="I79" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="J79" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K79" s="12" t="s">
         <v>255</v>
@@ -4886,10 +4886,10 @@
         <v>253</v>
       </c>
       <c r="I80" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="J80" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K80" s="12" t="s">
         <v>255</v>
@@ -4919,10 +4919,10 @@
         <v>253</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="J81" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K81" s="12" t="s">
         <v>255</v>
@@ -4952,7 +4952,7 @@
         <v>253</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J82" s="3" t="s">
         <v>254</v>
@@ -5044,7 +5044,7 @@
         <v>253</v>
       </c>
       <c r="I85" s="7" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J85" s="7" t="s">
         <v>254</v>
@@ -5076,7 +5076,7 @@
         <v>253</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J86" s="3" t="s">
         <v>254</v>
@@ -5108,7 +5108,7 @@
         <v>253</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J87" s="3" t="s">
         <v>254</v>
@@ -5140,7 +5140,7 @@
         <v>253</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J88" s="3" t="s">
         <v>254</v>
@@ -5173,7 +5173,7 @@
         <v>253</v>
       </c>
       <c r="I89" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J89" s="3" t="s">
         <v>254</v>
@@ -5206,7 +5206,7 @@
         <v>253</v>
       </c>
       <c r="I90" s="7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J90" s="3" t="s">
         <v>254</v>
@@ -5239,7 +5239,7 @@
         <v>253</v>
       </c>
       <c r="I91" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J91" s="3" t="s">
         <v>254</v>
@@ -5272,7 +5272,7 @@
         <v>253</v>
       </c>
       <c r="I92" s="14" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J92" s="3" t="s">
         <v>254</v>
@@ -5576,7 +5576,7 @@
         <v>253</v>
       </c>
       <c r="I102" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J102" s="3" t="s">
         <v>254</v>
@@ -5608,10 +5608,10 @@
         <v>253</v>
       </c>
       <c r="I103" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J103" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K103" s="3" t="s">
         <v>255</v>
@@ -5641,7 +5641,7 @@
         <v>253</v>
       </c>
       <c r="I104" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J104" s="3" t="s">
         <v>254</v>
@@ -5674,7 +5674,7 @@
         <v>253</v>
       </c>
       <c r="I105" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J105" s="3" t="s">
         <v>254</v>
@@ -5707,7 +5707,7 @@
         <v>253</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J106" s="3" t="s">
         <v>254</v>
@@ -5740,10 +5740,10 @@
         <v>253</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K107" s="3" t="s">
         <v>255</v>
@@ -5803,10 +5803,10 @@
         <v>253</v>
       </c>
       <c r="I109" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J109" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K109" s="3" t="s">
         <v>255</v>
@@ -5836,10 +5836,10 @@
         <v>253</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J110" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K110" s="3" t="s">
         <v>255</v>
@@ -5869,7 +5869,7 @@
         <v>253</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J111" s="3" t="s">
         <v>254</v>
@@ -5902,10 +5902,10 @@
         <v>253</v>
       </c>
       <c r="I112" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K112" s="3" t="s">
         <v>255</v>
@@ -5934,10 +5934,10 @@
         <v>253</v>
       </c>
       <c r="I113" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J113" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K113" s="3" t="s">
         <v>255</v>
@@ -5966,10 +5966,10 @@
         <v>253</v>
       </c>
       <c r="I114" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J114" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K114" s="3" t="s">
         <v>255</v>
@@ -6030,7 +6030,7 @@
         <v>253</v>
       </c>
       <c r="I116" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J116" s="3" t="s">
         <v>254</v>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="I117" s="5"/>
       <c r="J117" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K117" s="3" t="s">
         <v>255</v>
@@ -6173,16 +6173,16 @@
         <v>273</v>
       </c>
       <c r="F121" t="s">
+        <v>339</v>
+      </c>
+      <c r="G121" t="s">
         <v>274</v>
-      </c>
-      <c r="G121" t="s">
-        <v>275</v>
       </c>
       <c r="H121" s="8">
         <v>2</v>
       </c>
       <c r="I121" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J121" s="3" t="s">
         <v>254</v>

</xml_diff>